<commit_message>
Merged PR 1417: PROPH-1158-Comment-Export-Rework into UAT
Split Id's and Titles for the BOE, CLIN and WBS and added confirmation dialog as suggested by Immanuel.
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/CommentsAndResponses.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/CommentsAndResponses.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26130"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76D68032-2E53-4DE8-A4F0-09DB3D8829AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{317EC94C-0494-4980-BA77-9621199AC28E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,46 +24,7 @@
     <author>Author</author>
   </authors>
   <commentList>
-    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Id + Title of the BOE</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{20EAF21F-A4FF-41FA-9391-0E6EFD544245}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Clin Number + Clin Title</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{0AFAC7B2-A8DB-441F-B6B9-4755FD89AD37}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Wbs number + Title</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
+    <comment ref="G1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
       <text>
         <r>
           <rPr>
@@ -76,7 +37,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
+    <comment ref="I1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
       <text>
         <r>
           <rPr>
@@ -89,7 +50,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I1" authorId="0" shapeId="0" xr:uid="{518098F9-DF46-4F4A-9EE0-CE15A6F4C3D2}">
+    <comment ref="L1" authorId="0" shapeId="0" xr:uid="{518098F9-DF46-4F4A-9EE0-CE15A6F4C3D2}">
       <text>
         <r>
           <rPr>
@@ -107,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>ContractTypes</t>
   </si>
@@ -136,13 +97,22 @@
     <t>Author Response Timestamp</t>
   </si>
   <si>
-    <t>CLIN</t>
-  </si>
-  <si>
-    <t>WBS</t>
-  </si>
-  <si>
-    <t>BOE</t>
+    <t>BOE Title</t>
+  </si>
+  <si>
+    <t>BOE ID</t>
+  </si>
+  <si>
+    <t>CLIN Title</t>
+  </si>
+  <si>
+    <t>WBS #</t>
+  </si>
+  <si>
+    <t>WBS Title</t>
+  </si>
+  <si>
+    <t>CLIN #</t>
   </si>
 </sst>
 </file>
@@ -590,57 +560,71 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="3" width="27.140625" style="4" customWidth="1"/>
-    <col min="4" max="4" width="34.7109375" style="3" customWidth="1"/>
-    <col min="5" max="5" width="24.5703125" style="3" customWidth="1"/>
-    <col min="6" max="6" width="20.7109375" style="3" customWidth="1"/>
-    <col min="7" max="7" width="47.85546875" style="3" customWidth="1"/>
-    <col min="8" max="8" width="25.85546875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="22.42578125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="47.28515625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="29.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="17.7109375" style="4" customWidth="1"/>
+    <col min="2" max="2" width="27.140625" style="4" customWidth="1"/>
+    <col min="3" max="3" width="17.7109375" style="4" customWidth="1"/>
+    <col min="4" max="4" width="27.140625" style="4" customWidth="1"/>
+    <col min="5" max="5" width="17.7109375" style="4" customWidth="1"/>
+    <col min="6" max="6" width="27.140625" style="4" customWidth="1"/>
+    <col min="7" max="7" width="34.7109375" style="3" customWidth="1"/>
+    <col min="8" max="8" width="24.5703125" style="3" customWidth="1"/>
+    <col min="9" max="9" width="20.7109375" style="3" customWidth="1"/>
+    <col min="10" max="10" width="47.85546875" style="3" customWidth="1"/>
+    <col min="11" max="11" width="25.85546875" style="1" customWidth="1"/>
+    <col min="12" max="12" width="22.42578125" style="1" customWidth="1"/>
+    <col min="13" max="13" width="47.28515625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="29.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="2" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" s="2" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="13.5" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="1:14" ht="13.5" thickTop="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -668,12 +652,16 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <documentManagement>
+    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
+    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
+      <Value>2</Value>
+    </SipLabel>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -780,22 +768,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <documentManagement>
-    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
-    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
-      <Value>2</Value>
-    </SipLabel>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DCDA7760-8C18-4744-80BE-EC14AF3979C1}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E141511F-2C2D-45F4-A120-F9C297666AB6}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
+    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
+    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -820,18 +813,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E141511F-2C2D-45F4-A120-F9C297666AB6}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DCDA7760-8C18-4744-80BE-EC14AF3979C1}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
-    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
-    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>